<commit_message>
Sheets renamed: Chunks_Methodology and Chunks_Documentation
Chunks_Canon is now Chunks_Methodology and Chunks_Doc is Chunks_Documentation;
Chunks_Model is unchanged. Cell 4's re-reading checks name the sheets too. The
records behind them keep their names (chunks_canon, chunks_doc) and their
references (C-, D-), so the audit log of an earlier run still reads back.

Checked: all eight samples - every sheet's content identical, only the two
names changed; the manual names only sheets that exist; the notebook's four
cells ran and cell 4 confirmed all eight checks.
</commit_message>
<xml_diff>
--- a/Engine_Map.xlsx
+++ b/Engine_Map.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>5663 lines, 239 functions and classes, 64 sections</t>
+          <t>5664 lines, 239 functions and classes, 64 sections</t>
         </is>
       </c>
     </row>
@@ -11308,7 +11308,7 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>The rows of Chunks_Canon and Chunks_Doc.</t>
+          <t>The rows of Chunks_Methodology and Chunks_Documentation.</t>
         </is>
       </c>
       <c r="H215" s="3" t="inlineStr"/>
@@ -11841,11 +11841,11 @@
       </c>
       <c r="E226" s="3" t="inlineStr">
         <is>
-          <t>5363-5404</t>
+          <t>5363-5405</t>
         </is>
       </c>
       <c r="F226" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G226" s="3" t="inlineStr">
         <is>
@@ -11892,7 +11892,7 @@
       </c>
       <c r="E227" s="3" t="inlineStr">
         <is>
-          <t>5406-5422</t>
+          <t>5407-5423</t>
         </is>
       </c>
       <c r="F227" s="3" t="n">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="E228" s="3" t="inlineStr">
         <is>
-          <t>5424-5427</t>
+          <t>5425-5428</t>
         </is>
       </c>
       <c r="F228" s="3" t="n">
@@ -11990,7 +11990,7 @@
       </c>
       <c r="E229" s="3" t="inlineStr">
         <is>
-          <t>5429-5431</t>
+          <t>5430-5432</t>
         </is>
       </c>
       <c r="F229" s="3" t="n">
@@ -12037,7 +12037,7 @@
       </c>
       <c r="E230" s="3" t="inlineStr">
         <is>
-          <t>5455-5469</t>
+          <t>5456-5470</t>
         </is>
       </c>
       <c r="F230" s="3" t="n">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="E231" s="3" t="inlineStr">
         <is>
-          <t>5471-5480</t>
+          <t>5472-5481</t>
         </is>
       </c>
       <c r="F231" s="3" t="n">
@@ -12135,7 +12135,7 @@
       </c>
       <c r="E232" s="3" t="inlineStr">
         <is>
-          <t>5482-5487</t>
+          <t>5483-5488</t>
         </is>
       </c>
       <c r="F232" s="3" t="n">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="E233" s="3" t="inlineStr">
         <is>
-          <t>5489-5531</t>
+          <t>5490-5532</t>
         </is>
       </c>
       <c r="F233" s="3" t="n">
@@ -12229,7 +12229,7 @@
       </c>
       <c r="E234" s="3" t="inlineStr">
         <is>
-          <t>5533-5542</t>
+          <t>5534-5543</t>
         </is>
       </c>
       <c r="F234" s="3" t="n">
@@ -12276,7 +12276,7 @@
       </c>
       <c r="E235" s="3" t="inlineStr">
         <is>
-          <t>5544-5586</t>
+          <t>5545-5587</t>
         </is>
       </c>
       <c r="F235" s="3" t="n">
@@ -12327,7 +12327,7 @@
       </c>
       <c r="E236" s="3" t="inlineStr">
         <is>
-          <t>5588-5589</t>
+          <t>5589-5590</t>
         </is>
       </c>
       <c r="F236" s="3" t="n">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="E237" s="3" t="inlineStr">
         <is>
-          <t>5591-5612</t>
+          <t>5592-5613</t>
         </is>
       </c>
       <c r="F237" s="3" t="n">
@@ -12425,7 +12425,7 @@
       </c>
       <c r="E238" s="3" t="inlineStr">
         <is>
-          <t>5614-5627</t>
+          <t>5615-5628</t>
         </is>
       </c>
       <c r="F238" s="3" t="n">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="E239" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="F239" s="3" t="n">
@@ -12527,7 +12527,7 @@
       </c>
       <c r="E240" s="3" t="inlineStr">
         <is>
-          <t>5652-5662</t>
+          <t>5653-5663</t>
         </is>
       </c>
       <c r="F240" s="3" t="n">
@@ -13464,7 +13464,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>5424-5427</t>
+          <t>5425-5428</t>
         </is>
       </c>
       <c r="P11" s="3" t="n">
@@ -13521,7 +13521,7 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>5406-5422</t>
+          <t>5407-5423</t>
         </is>
       </c>
       <c r="P12" s="3" t="n">
@@ -20606,7 +20606,7 @@
       </c>
       <c r="O109" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P109" s="3" t="n">
@@ -20691,7 +20691,7 @@
       </c>
       <c r="O110" s="3" t="inlineStr">
         <is>
-          <t>5588-5589</t>
+          <t>5589-5590</t>
         </is>
       </c>
       <c r="P110" s="3" t="n">
@@ -20861,7 +20861,7 @@
       </c>
       <c r="O112" s="3" t="inlineStr">
         <is>
-          <t>5614-5627</t>
+          <t>5615-5628</t>
         </is>
       </c>
       <c r="P112" s="3" t="n">
@@ -23159,7 +23159,7 @@
       </c>
       <c r="O138" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P138" s="3" t="n">
@@ -23252,7 +23252,7 @@
       </c>
       <c r="O139" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P139" s="3" t="n">
@@ -24045,7 +24045,7 @@
       </c>
       <c r="Q148" s="3" t="inlineStr">
         <is>
-          <t>The rows of Chunks_Canon and Chunks_Doc.</t>
+          <t>The rows of Chunks_Methodology and Chunks_Documentation.</t>
         </is>
       </c>
       <c r="R148" s="3" t="inlineStr"/>
@@ -26505,7 +26505,7 @@
       </c>
       <c r="O176" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P176" s="3" t="n">
@@ -39013,7 +39013,7 @@
       </c>
       <c r="O328" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P328" s="3" t="n">
@@ -45138,7 +45138,7 @@
       </c>
       <c r="O413" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P413" s="3" t="n">
@@ -45973,7 +45973,7 @@
       </c>
       <c r="O424" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P424" s="3" t="n">
@@ -50373,7 +50373,7 @@
       </c>
       <c r="O488" s="3" t="inlineStr">
         <is>
-          <t>5429-5431</t>
+          <t>5430-5432</t>
         </is>
       </c>
       <c r="P488" s="3" t="n">
@@ -51316,7 +51316,7 @@
       </c>
       <c r="O503" s="3" t="inlineStr">
         <is>
-          <t>5489-5531</t>
+          <t>5490-5532</t>
         </is>
       </c>
       <c r="P503" s="3" t="n">
@@ -51373,7 +51373,7 @@
       </c>
       <c r="O504" s="3" t="inlineStr">
         <is>
-          <t>5455-5469</t>
+          <t>5456-5470</t>
         </is>
       </c>
       <c r="P504" s="3" t="n">
@@ -51487,7 +51487,7 @@
       </c>
       <c r="O506" s="3" t="inlineStr">
         <is>
-          <t>5544-5586</t>
+          <t>5545-5587</t>
         </is>
       </c>
       <c r="P506" s="3" t="n">
@@ -51548,7 +51548,7 @@
       </c>
       <c r="O507" s="3" t="inlineStr">
         <is>
-          <t>5533-5542</t>
+          <t>5534-5543</t>
         </is>
       </c>
       <c r="P507" s="3" t="n">
@@ -51601,7 +51601,7 @@
       </c>
       <c r="O508" s="3" t="inlineStr">
         <is>
-          <t>5471-5480</t>
+          <t>5472-5481</t>
         </is>
       </c>
       <c r="P508" s="3" t="n">
@@ -51727,7 +51727,7 @@
       </c>
       <c r="O510" s="3" t="inlineStr">
         <is>
-          <t>5471-5480</t>
+          <t>5472-5481</t>
         </is>
       </c>
       <c r="P510" s="3" t="n">
@@ -51788,7 +51788,7 @@
       </c>
       <c r="O511" s="3" t="inlineStr">
         <is>
-          <t>5482-5487</t>
+          <t>5483-5488</t>
         </is>
       </c>
       <c r="P511" s="3" t="n">
@@ -51841,7 +51841,7 @@
       </c>
       <c r="O512" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P512" s="3" t="n">
@@ -51898,7 +51898,7 @@
       </c>
       <c r="O513" s="3" t="inlineStr">
         <is>
-          <t>5591-5612</t>
+          <t>5592-5613</t>
         </is>
       </c>
       <c r="P513" s="3" t="n">
@@ -52012,7 +52012,7 @@
       </c>
       <c r="O515" s="3" t="inlineStr">
         <is>
-          <t>5629-5650</t>
+          <t>5630-5651</t>
         </is>
       </c>
       <c r="P515" s="3" t="n">
@@ -52069,7 +52069,7 @@
       </c>
       <c r="O516" s="3" t="inlineStr">
         <is>
-          <t>5652-5662</t>
+          <t>5653-5663</t>
         </is>
       </c>
       <c r="P516" s="3" t="n">
@@ -52187,7 +52187,7 @@
       </c>
       <c r="O518" s="3" t="inlineStr">
         <is>
-          <t>5471-5480</t>
+          <t>5472-5481</t>
         </is>
       </c>
       <c r="P518" s="3" t="n">
@@ -52248,7 +52248,7 @@
       </c>
       <c r="O519" s="3" t="inlineStr">
         <is>
-          <t>5588-5589</t>
+          <t>5589-5590</t>
         </is>
       </c>
       <c r="P519" s="3" t="n">
@@ -52309,11 +52309,11 @@
       </c>
       <c r="O520" s="3" t="inlineStr">
         <is>
-          <t>5363-5404</t>
+          <t>5363-5405</t>
         </is>
       </c>
       <c r="P520" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q520" s="3" t="inlineStr">
         <is>
@@ -52817,7 +52817,7 @@
       </c>
       <c r="O528" s="3" t="inlineStr">
         <is>
-          <t>5471-5480</t>
+          <t>5472-5481</t>
         </is>
       </c>
       <c r="P528" s="3" t="n">
@@ -53191,7 +53191,7 @@
       </c>
       <c r="O534" s="3" t="inlineStr">
         <is>
-          <t>5471-5480</t>
+          <t>5472-5481</t>
         </is>
       </c>
       <c r="P534" s="3" t="n">
@@ -55037,7 +55037,7 @@
         <v>5343</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>5</v>
@@ -55055,7 +55055,7 @@
         </is>
       </c>
       <c r="B65" s="3" t="n">
-        <v>5443</v>
+        <v>5444</v>
       </c>
       <c r="C65" s="3" t="n">
         <v>221</v>

</xml_diff>